<commit_message>
Fix PO template v3: zebra on calculated cols, white input cols, empty defaults, complete logo border, band borders
</commit_message>
<xml_diff>
--- a/app/public/templates/Purchase_Order_Template_v2.xlsx
+++ b/app/public/templates/Purchase_Order_Template_v2.xlsx
@@ -154,7 +154,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -172,8 +172,8 @@
       <top style="dashed">
         <color rgb="FF9CA3AF"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFE5E7EB"/>
+      <bottom style="dashed">
+        <color rgb="FF9CA3AF"/>
       </bottom>
     </border>
     <border>
@@ -218,26 +218,33 @@
         <color rgb="FF9CA3AF"/>
       </bottom>
     </border>
+    <border/>
     <border>
+      <left style="thin">
+        <color rgb="FF9CA3AF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9CA3AF"/>
+      </right>
       <top style="thin">
         <color rgb="FF9CA3AF"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFE5E7EB"/>
-      </bottom>
     </border>
     <border>
-      <top style="thin">
-        <color rgb="FFE5E7EB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFE5E7EB"/>
-      </bottom>
+      <left style="thin">
+        <color rgb="FF9CA3AF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9CA3AF"/>
+      </right>
     </border>
     <border>
-      <top style="thin">
-        <color rgb="FFE5E7EB"/>
-      </top>
+      <left style="thin">
+        <color rgb="FF9CA3AF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9CA3AF"/>
+      </right>
       <bottom style="thin">
         <color rgb="FF9CA3AF"/>
       </bottom>
@@ -285,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -298,48 +305,44 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -356,10 +359,13 @@
     <xf numFmtId="9" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -368,23 +374,23 @@
     <xf numFmtId="166" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -806,207 +812,193 @@
           <t>Supplier name</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>ORDER DATE</t>
         </is>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="8">
         <f>DATE(2026,6,18)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="18.95" customHeight="1">
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>REQUIRED BY</t>
         </is>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="8">
         <f>DATE(2026,7,2)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="18.95" customHeight="1">
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Town / City</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>BUYER</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Buyer name</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18.95" customHeight="1">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>County</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>DELIVERY TERMS</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>e.g. FOB / Delivered</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18.95" customHeight="1">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Postcode</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18.95" customHeight="1">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18.95" customHeight="1">
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15.95" customHeight="1">
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>PO NO.</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>ORDER DATE</t>
         </is>
       </c>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>REQUIRED BY</t>
         </is>
       </c>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="16" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>ORDER TOTAL</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="17">
+      <c r="B16" s="14">
         <f>G6</f>
         <v/>
       </c>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="17">
+      <c r="D16" s="14">
         <f>G7</f>
         <v/>
       </c>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="17">
+      <c r="F16" s="14">
         <f>G8</f>
         <v/>
       </c>
-      <c r="G16" s="15" t="n"/>
-      <c r="H16" s="18">
+      <c r="H16" s="15">
         <f>H33</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Description / Part</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>Unit price</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="F18" s="20" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>VAT %</t>
         </is>
       </c>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="G18" s="18" t="inlineStr">
         <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="H18" s="20" t="inlineStr">
+      <c r="H18" s="18" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20.1" customHeight="1">
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="24">
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="22">
         <f>IF(AND(C19="",D19=""),"",C19*D19)</f>
         <v/>
       </c>
-      <c r="F19" s="25" t="n">
+      <c r="F19" s="23" t="n">
         <v>0.05</v>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="22">
         <f>IF(E19="","",E19*F19)</f>
         <v/>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="22">
         <f>IF(E19="","",E19+G19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="20.1" customHeight="1">
-      <c r="B20" s="21" t="n"/>
-      <c r="C20" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="20" t="n"/>
+      <c r="D20" s="21" t="n"/>
       <c r="E20" s="24">
         <f>IF(AND(C20="",D20=""),"",C20*D20)</f>
         <v/>
       </c>
-      <c r="F20" s="25" t="n">
+      <c r="F20" s="23" t="n">
         <v>0.2</v>
       </c>
       <c r="G20" s="24">
@@ -1019,42 +1011,34 @@
       </c>
     </row>
     <row r="21" ht="20.1" customHeight="1">
-      <c r="B21" s="21" t="n"/>
-      <c r="C21" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="24">
+      <c r="B21" s="19" t="n"/>
+      <c r="C21" s="20" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="22">
         <f>IF(AND(C21="",D21=""),"",C21*D21)</f>
         <v/>
       </c>
-      <c r="F21" s="25" t="n">
+      <c r="F21" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="G21" s="24">
+      <c r="G21" s="22">
         <f>IF(E21="","",E21*F21)</f>
         <v/>
       </c>
-      <c r="H21" s="24">
+      <c r="H21" s="22">
         <f>IF(E21="","",E21+G21)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="20.1" customHeight="1">
-      <c r="B22" s="21" t="n"/>
-      <c r="C22" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="20" t="n"/>
+      <c r="D22" s="21" t="n"/>
       <c r="E22" s="24">
         <f>IF(AND(C22="",D22=""),"",C22*D22)</f>
         <v/>
       </c>
-      <c r="F22" s="25" t="n">
+      <c r="F22" s="23" t="n">
         <v>0.2</v>
       </c>
       <c r="G22" s="24">
@@ -1067,42 +1051,34 @@
       </c>
     </row>
     <row r="23" ht="20.1" customHeight="1">
-      <c r="B23" s="21" t="n"/>
-      <c r="C23" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="24">
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="20" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="22">
         <f>IF(AND(C23="",D23=""),"",C23*D23)</f>
         <v/>
       </c>
-      <c r="F23" s="25" t="n">
+      <c r="F23" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="G23" s="24">
+      <c r="G23" s="22">
         <f>IF(E23="","",E23*F23)</f>
         <v/>
       </c>
-      <c r="H23" s="24">
+      <c r="H23" s="22">
         <f>IF(E23="","",E23+G23)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="20.1" customHeight="1">
-      <c r="B24" s="21" t="n"/>
-      <c r="C24" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="20" t="n"/>
+      <c r="D24" s="21" t="n"/>
       <c r="E24" s="24">
         <f>IF(AND(C24="",D24=""),"",C24*D24)</f>
         <v/>
       </c>
-      <c r="F24" s="25" t="n">
+      <c r="F24" s="23" t="n">
         <v>0.2</v>
       </c>
       <c r="G24" s="24">
@@ -1115,42 +1091,34 @@
       </c>
     </row>
     <row r="25" ht="20.1" customHeight="1">
-      <c r="B25" s="21" t="n"/>
-      <c r="C25" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="24">
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="22">
         <f>IF(AND(C25="",D25=""),"",C25*D25)</f>
         <v/>
       </c>
-      <c r="F25" s="25" t="n">
+      <c r="F25" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="22">
         <f>IF(E25="","",E25*F25)</f>
         <v/>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="22">
         <f>IF(E25="","",E25+G25)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="20.1" customHeight="1">
-      <c r="B26" s="21" t="n"/>
-      <c r="C26" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="21" t="n"/>
       <c r="E26" s="24">
         <f>IF(AND(C26="",D26=""),"",C26*D26)</f>
         <v/>
       </c>
-      <c r="F26" s="25" t="n">
+      <c r="F26" s="23" t="n">
         <v>0.2</v>
       </c>
       <c r="G26" s="24">
@@ -1163,42 +1131,34 @@
       </c>
     </row>
     <row r="27" ht="20.1" customHeight="1">
-      <c r="B27" s="21" t="n"/>
-      <c r="C27" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="24">
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="22">
         <f>IF(AND(C27="",D27=""),"",C27*D27)</f>
         <v/>
       </c>
-      <c r="F27" s="25" t="n">
+      <c r="F27" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="22">
         <f>IF(E27="","",E27*F27)</f>
         <v/>
       </c>
-      <c r="H27" s="24">
+      <c r="H27" s="22">
         <f>IF(E27="","",E27+G27)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="20.1" customHeight="1">
-      <c r="B28" s="21" t="n"/>
-      <c r="C28" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="21" t="n"/>
       <c r="E28" s="24">
         <f>IF(AND(C28="",D28=""),"",C28*D28)</f>
         <v/>
       </c>
-      <c r="F28" s="25" t="n">
+      <c r="F28" s="23" t="n">
         <v>0.2</v>
       </c>
       <c r="G28" s="24">
@@ -1211,42 +1171,34 @@
       </c>
     </row>
     <row r="29" ht="20.1" customHeight="1">
-      <c r="B29" s="21" t="n"/>
-      <c r="C29" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="24">
+      <c r="B29" s="19" t="n"/>
+      <c r="C29" s="20" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="22">
         <f>IF(AND(C29="",D29=""),"",C29*D29)</f>
         <v/>
       </c>
-      <c r="F29" s="25" t="n">
+      <c r="F29" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="G29" s="24">
+      <c r="G29" s="22">
         <f>IF(E29="","",E29*F29)</f>
         <v/>
       </c>
-      <c r="H29" s="24">
+      <c r="H29" s="22">
         <f>IF(E29="","",E29+G29)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="20.1" customHeight="1">
-      <c r="B30" s="21" t="n"/>
-      <c r="C30" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="21" t="n"/>
       <c r="E30" s="24">
         <f>IF(AND(C30="",D30=""),"",C30*D30)</f>
         <v/>
       </c>
-      <c r="F30" s="25" t="n">
+      <c r="F30" s="23" t="n">
         <v>0.2</v>
       </c>
       <c r="G30" s="24">
@@ -1259,34 +1211,34 @@
       </c>
     </row>
     <row r="31">
-      <c r="F31" s="26" t="inlineStr">
+      <c r="F31" s="25" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="H31" s="27">
+      <c r="H31" s="26">
         <f>SUM(E19:E30)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="F32" s="28" t="inlineStr">
+      <c r="F32" s="27" t="inlineStr">
         <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="H32" s="29">
+      <c r="H32" s="28">
         <f>SUM(G19:G30)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="F33" s="30" t="inlineStr">
+      <c r="F33" s="29" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="H33" s="31">
+      <c r="H33" s="30">
         <f>H31+H32</f>
         <v/>
       </c>
@@ -1297,38 +1249,38 @@
           <t>NOTES</t>
         </is>
       </c>
-      <c r="F35" s="32" t="inlineStr">
+      <c r="F35" s="31" t="inlineStr">
         <is>
           <t>Issued by, signature:</t>
         </is>
       </c>
     </row>
     <row r="36" ht="21.95" customHeight="1">
-      <c r="B36" s="33" t="inlineStr">
+      <c r="B36" s="32" t="inlineStr">
         <is>
           <t>Delivery instructions, references, special terms…</t>
         </is>
       </c>
-      <c r="F36" s="34" t="n"/>
+      <c r="F36" s="33" t="n"/>
     </row>
     <row r="37"/>
     <row r="38"/>
     <row r="40" ht="18" customHeight="1">
-      <c r="B40" s="35" t="inlineStr">
+      <c r="B40" s="34" t="inlineStr">
         <is>
           <t>Your Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15.95" customHeight="1">
-      <c r="B41" s="36" t="inlineStr">
+      <c r="B41" s="35" t="inlineStr">
         <is>
           <t>123 Example Street, London, EC1A 1BB</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15.95" customHeight="1">
-      <c r="B42" s="36" t="inlineStr">
+      <c r="B42" s="35" t="inlineStr">
         <is>
           <t>Tel 020 0000 0000   ·   accounts@yourcompany.co.uk   ·   VAT Reg GB000000000</t>
         </is>

</xml_diff>